<commit_message>
generated results for new30 - gpt4o but struggling with merging due to QID mapping issues
</commit_message>
<xml_diff>
--- a/eval/learning-curve/results/learning_curve_llama3.1-70b_ft200_incorrect.xlsx
+++ b/eval/learning-curve/results/learning_curve_llama3.1-70b_ft200_incorrect.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E345"/>
+  <dimension ref="A1:E550"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8983,6 +8983,4311 @@
         <v>0</v>
       </c>
     </row>
+    <row r="346">
+      <c r="A346" t="inlineStr">
+        <is>
+          <t>40391923</t>
+        </is>
+      </c>
+      <c r="B346" t="inlineStr">
+        <is>
+          <t>Does the paper report HIV sequences from patient samples?</t>
+        </is>
+      </c>
+      <c r="C346" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D346" t="inlineStr"/>
+      <c r="E346" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="347">
+      <c r="A347" t="inlineStr">
+        <is>
+          <t>40391923</t>
+        </is>
+      </c>
+      <c r="B347" t="inlineStr">
+        <is>
+          <t>What were the GenBank accession numbers for sequenced HIV isolates?</t>
+        </is>
+      </c>
+      <c r="C347" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D347" t="inlineStr"/>
+      <c r="E347" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="348">
+      <c r="A348" t="inlineStr">
+        <is>
+          <t>40391923</t>
+        </is>
+      </c>
+      <c r="B348" t="inlineStr">
+        <is>
+          <t>Which HIV genes were reported to have been sequenced?</t>
+        </is>
+      </c>
+      <c r="C348" t="inlineStr">
+        <is>
+          <t>PV008448-PV008641, PV407014-PV407203,  PV419497-PV419583</t>
+        </is>
+      </c>
+      <c r="D348" t="inlineStr"/>
+      <c r="E348" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="349">
+      <c r="A349" t="inlineStr">
+        <is>
+          <t>40391923</t>
+        </is>
+      </c>
+      <c r="B349" t="inlineStr">
+        <is>
+          <t>From which countries were the sequenced samples obtained?</t>
+        </is>
+      </c>
+      <c r="C349" t="inlineStr">
+        <is>
+          <t>227</t>
+        </is>
+      </c>
+      <c r="D349" t="inlineStr"/>
+      <c r="E349" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="350">
+      <c r="A350" t="inlineStr">
+        <is>
+          <t>40391923</t>
+        </is>
+      </c>
+      <c r="B350" t="inlineStr">
+        <is>
+          <t>From what years were the sequenced samples obtained?</t>
+        </is>
+      </c>
+      <c r="C350" t="inlineStr">
+        <is>
+          <t>Cameroon, Cote d'Ivoire, Malawi, Republic of Congo, Uganda, Zambia, Zimbabwe</t>
+        </is>
+      </c>
+      <c r="D350" t="inlineStr"/>
+      <c r="E350" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="351">
+      <c r="A351" t="inlineStr">
+        <is>
+          <t>40391923</t>
+        </is>
+      </c>
+      <c r="B351" t="inlineStr">
+        <is>
+          <t>What method was used for sequencing?</t>
+        </is>
+      </c>
+      <c r="C351" t="inlineStr">
+        <is>
+          <t>2022-2024</t>
+        </is>
+      </c>
+      <c r="D351" t="inlineStr"/>
+      <c r="E351" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="352">
+      <c r="A352" t="inlineStr">
+        <is>
+          <t>40391923</t>
+        </is>
+      </c>
+      <c r="B352" t="inlineStr">
+        <is>
+          <t>What type of samples were sequenced?</t>
+        </is>
+      </c>
+      <c r="C352" t="inlineStr">
+        <is>
+          <t>IN</t>
+        </is>
+      </c>
+      <c r="D352" t="inlineStr"/>
+      <c r="E352" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="353">
+      <c r="A353" t="inlineStr">
+        <is>
+          <t>40391923</t>
+        </is>
+      </c>
+      <c r="B353" t="inlineStr">
+        <is>
+          <t>How many individuals had samples obtained for HIV sequencing?</t>
+        </is>
+      </c>
+      <c r="C353" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D353" t="inlineStr"/>
+      <c r="E353" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="354">
+      <c r="A354" t="inlineStr">
+        <is>
+          <t>40391923</t>
+        </is>
+      </c>
+      <c r="B354" t="inlineStr">
+        <is>
+          <t>Which drug classes were received by individuals in the study before sample sequencing?</t>
+        </is>
+      </c>
+      <c r="C354" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D354" t="inlineStr"/>
+      <c r="E354" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="355">
+      <c r="A355" t="inlineStr">
+        <is>
+          <t>40391923</t>
+        </is>
+      </c>
+      <c r="B355" t="inlineStr">
+        <is>
+          <t>Which drugs were received by individuals in the study before sample sequencing?</t>
+        </is>
+      </c>
+      <c r="C355" t="inlineStr">
+        <is>
+          <t>NRTI, NNRTI, INSTI</t>
+        </is>
+      </c>
+      <c r="D355" t="inlineStr"/>
+      <c r="E355" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="356">
+      <c r="A356" t="inlineStr">
+        <is>
+          <t>40400229</t>
+        </is>
+      </c>
+      <c r="B356" t="inlineStr">
+        <is>
+          <t>Does the paper report HIV sequences from patient samples?</t>
+        </is>
+      </c>
+      <c r="C356" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D356" t="inlineStr"/>
+      <c r="E356" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="357">
+      <c r="A357" t="inlineStr">
+        <is>
+          <t>40400229</t>
+        </is>
+      </c>
+      <c r="B357" t="inlineStr">
+        <is>
+          <t>From which countries were the sequenced samples obtained?</t>
+        </is>
+      </c>
+      <c r="C357" t="inlineStr">
+        <is>
+          <t>47</t>
+        </is>
+      </c>
+      <c r="D357" t="inlineStr"/>
+      <c r="E357" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="358">
+      <c r="A358" t="inlineStr">
+        <is>
+          <t>40400229</t>
+        </is>
+      </c>
+      <c r="B358" t="inlineStr">
+        <is>
+          <t>From what years were the sequenced samples obtained?</t>
+        </is>
+      </c>
+      <c r="C358" t="inlineStr">
+        <is>
+          <t>UK</t>
+        </is>
+      </c>
+      <c r="D358" t="inlineStr"/>
+      <c r="E358" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="359">
+      <c r="A359" t="inlineStr">
+        <is>
+          <t>40400229</t>
+        </is>
+      </c>
+      <c r="B359" t="inlineStr">
+        <is>
+          <t>What method was used for sequencing?</t>
+        </is>
+      </c>
+      <c r="C359" t="inlineStr">
+        <is>
+          <t>2017-2020</t>
+        </is>
+      </c>
+      <c r="D359" t="inlineStr"/>
+      <c r="E359" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="360">
+      <c r="A360" t="inlineStr">
+        <is>
+          <t>40400229</t>
+        </is>
+      </c>
+      <c r="B360" t="inlineStr">
+        <is>
+          <t>What type of samples were sequenced?</t>
+        </is>
+      </c>
+      <c r="C360" t="inlineStr">
+        <is>
+          <t>RT,IN</t>
+        </is>
+      </c>
+      <c r="D360" t="inlineStr"/>
+      <c r="E360" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="361">
+      <c r="A361" t="inlineStr">
+        <is>
+          <t>40400229</t>
+        </is>
+      </c>
+      <c r="B361" t="inlineStr">
+        <is>
+          <t>How many individuals had samples obtained for HIV sequencing?</t>
+        </is>
+      </c>
+      <c r="C361" t="inlineStr">
+        <is>
+          <t>Yes (PrEP)</t>
+        </is>
+      </c>
+      <c r="D361" t="inlineStr"/>
+      <c r="E361" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="362">
+      <c r="A362" t="inlineStr">
+        <is>
+          <t>40400229</t>
+        </is>
+      </c>
+      <c r="B362" t="inlineStr">
+        <is>
+          <t>Which drug classes were received by individuals in the study before sample sequencing?</t>
+        </is>
+      </c>
+      <c r="C362" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D362" t="inlineStr"/>
+      <c r="E362" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="363">
+      <c r="A363" t="inlineStr">
+        <is>
+          <t>40400229</t>
+        </is>
+      </c>
+      <c r="B363" t="inlineStr">
+        <is>
+          <t>Which drugs were received by individuals in the study before sample sequencing?</t>
+        </is>
+      </c>
+      <c r="C363" t="inlineStr">
+        <is>
+          <t>RT</t>
+        </is>
+      </c>
+      <c r="D363" t="inlineStr"/>
+      <c r="E363" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="364">
+      <c r="A364" t="inlineStr">
+        <is>
+          <t>40431710</t>
+        </is>
+      </c>
+      <c r="B364" t="inlineStr">
+        <is>
+          <t>Does the paper report HIV sequences from patient samples?</t>
+        </is>
+      </c>
+      <c r="C364" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D364" t="inlineStr"/>
+      <c r="E364" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="365">
+      <c r="A365" t="inlineStr">
+        <is>
+          <t>40431710</t>
+        </is>
+      </c>
+      <c r="B365" t="inlineStr">
+        <is>
+          <t>From which countries were the sequenced samples obtained?</t>
+        </is>
+      </c>
+      <c r="C365" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D365" t="inlineStr"/>
+      <c r="E365" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="366">
+      <c r="A366" t="inlineStr">
+        <is>
+          <t>40431710</t>
+        </is>
+      </c>
+      <c r="B366" t="inlineStr">
+        <is>
+          <t>From what years were the sequenced samples obtained?</t>
+        </is>
+      </c>
+      <c r="C366" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="D366" t="inlineStr"/>
+      <c r="E366" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="367">
+      <c r="A367" t="inlineStr">
+        <is>
+          <t>40431710</t>
+        </is>
+      </c>
+      <c r="B367" t="inlineStr">
+        <is>
+          <t>What method was used for sequencing?</t>
+        </is>
+      </c>
+      <c r="C367" t="inlineStr">
+        <is>
+          <t>2006-2024</t>
+        </is>
+      </c>
+      <c r="D367" t="inlineStr"/>
+      <c r="E367" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="368">
+      <c r="A368" t="inlineStr">
+        <is>
+          <t>40431710</t>
+        </is>
+      </c>
+      <c r="B368" t="inlineStr">
+        <is>
+          <t>What type of samples were sequenced?</t>
+        </is>
+      </c>
+      <c r="C368" t="inlineStr">
+        <is>
+          <t>RT, PR, IN</t>
+        </is>
+      </c>
+      <c r="D368" t="inlineStr"/>
+      <c r="E368" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="369">
+      <c r="A369" t="inlineStr">
+        <is>
+          <t>40431710</t>
+        </is>
+      </c>
+      <c r="B369" t="inlineStr">
+        <is>
+          <t>How many individuals had samples obtained for HIV sequencing?</t>
+        </is>
+      </c>
+      <c r="C369" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D369" t="inlineStr"/>
+      <c r="E369" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="370">
+      <c r="A370" t="inlineStr">
+        <is>
+          <t>40431710</t>
+        </is>
+      </c>
+      <c r="B370" t="inlineStr">
+        <is>
+          <t>Which drug classes were received by individuals in the study before sample sequencing?</t>
+        </is>
+      </c>
+      <c r="C370" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D370" t="inlineStr"/>
+      <c r="E370" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="371">
+      <c r="A371" t="inlineStr">
+        <is>
+          <t>40431710</t>
+        </is>
+      </c>
+      <c r="B371" t="inlineStr">
+        <is>
+          <t>Which drugs were received by individuals in the study before sample sequencing?</t>
+        </is>
+      </c>
+      <c r="C371" t="inlineStr">
+        <is>
+          <t>NRTI, NNRTI, PI, INSTI</t>
+        </is>
+      </c>
+      <c r="D371" t="inlineStr"/>
+      <c r="E371" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="372">
+      <c r="A372" t="inlineStr">
+        <is>
+          <t>40431742</t>
+        </is>
+      </c>
+      <c r="B372" t="inlineStr">
+        <is>
+          <t>Does the paper report HIV sequences from patient samples?</t>
+        </is>
+      </c>
+      <c r="C372" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D372" t="inlineStr"/>
+      <c r="E372" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="373">
+      <c r="A373" t="inlineStr">
+        <is>
+          <t>40431742</t>
+        </is>
+      </c>
+      <c r="B373" t="inlineStr">
+        <is>
+          <t>From which countries were the sequenced samples obtained?</t>
+        </is>
+      </c>
+      <c r="C373" t="inlineStr">
+        <is>
+          <t>1677</t>
+        </is>
+      </c>
+      <c r="D373" t="inlineStr"/>
+      <c r="E373" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="374">
+      <c r="A374" t="inlineStr">
+        <is>
+          <t>40431742</t>
+        </is>
+      </c>
+      <c r="B374" t="inlineStr">
+        <is>
+          <t>From what years were the sequenced samples obtained?</t>
+        </is>
+      </c>
+      <c r="C374" t="inlineStr">
+        <is>
+          <t>Argentina</t>
+        </is>
+      </c>
+      <c r="D374" t="inlineStr"/>
+      <c r="E374" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="375">
+      <c r="A375" t="inlineStr">
+        <is>
+          <t>40431742</t>
+        </is>
+      </c>
+      <c r="B375" t="inlineStr">
+        <is>
+          <t>What method was used for sequencing?</t>
+        </is>
+      </c>
+      <c r="C375" t="inlineStr">
+        <is>
+          <t>2017-2021</t>
+        </is>
+      </c>
+      <c r="D375" t="inlineStr"/>
+      <c r="E375" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="376">
+      <c r="A376" t="inlineStr">
+        <is>
+          <t>40431742</t>
+        </is>
+      </c>
+      <c r="B376" t="inlineStr">
+        <is>
+          <t>What type of samples were sequenced?</t>
+        </is>
+      </c>
+      <c r="C376" t="inlineStr">
+        <is>
+          <t>RT,PR</t>
+        </is>
+      </c>
+      <c r="D376" t="inlineStr"/>
+      <c r="E376" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="377">
+      <c r="A377" t="inlineStr">
+        <is>
+          <t>40490983</t>
+        </is>
+      </c>
+      <c r="B377" t="inlineStr">
+        <is>
+          <t>Does the paper report HIV sequences from patient samples?</t>
+        </is>
+      </c>
+      <c r="C377" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D377" t="inlineStr"/>
+      <c r="E377" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="378">
+      <c r="A378" t="inlineStr">
+        <is>
+          <t>40490983</t>
+        </is>
+      </c>
+      <c r="B378" t="inlineStr">
+        <is>
+          <t>From which countries were the sequenced samples obtained?</t>
+        </is>
+      </c>
+      <c r="C378" t="inlineStr">
+        <is>
+          <t>187</t>
+        </is>
+      </c>
+      <c r="D378" t="inlineStr"/>
+      <c r="E378" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="379">
+      <c r="A379" t="inlineStr">
+        <is>
+          <t>40490983</t>
+        </is>
+      </c>
+      <c r="B379" t="inlineStr">
+        <is>
+          <t>From what years were the sequenced samples obtained?</t>
+        </is>
+      </c>
+      <c r="C379" t="inlineStr">
+        <is>
+          <t>Kenya</t>
+        </is>
+      </c>
+      <c r="D379" t="inlineStr"/>
+      <c r="E379" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="380">
+      <c r="A380" t="inlineStr">
+        <is>
+          <t>40490983</t>
+        </is>
+      </c>
+      <c r="B380" t="inlineStr">
+        <is>
+          <t>What method was used for sequencing?</t>
+        </is>
+      </c>
+      <c r="C380" t="inlineStr">
+        <is>
+          <t>2011-2021</t>
+        </is>
+      </c>
+      <c r="D380" t="inlineStr"/>
+      <c r="E380" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="381">
+      <c r="A381" t="inlineStr">
+        <is>
+          <t>40490983</t>
+        </is>
+      </c>
+      <c r="B381" t="inlineStr">
+        <is>
+          <t>What type of samples were sequenced?</t>
+        </is>
+      </c>
+      <c r="C381" t="inlineStr">
+        <is>
+          <t>RT, PR</t>
+        </is>
+      </c>
+      <c r="D381" t="inlineStr"/>
+      <c r="E381" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="382">
+      <c r="A382" t="inlineStr">
+        <is>
+          <t>40490983</t>
+        </is>
+      </c>
+      <c r="B382" t="inlineStr">
+        <is>
+          <t>How many individuals had samples obtained for HIV sequencing?</t>
+        </is>
+      </c>
+      <c r="C382" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D382" t="inlineStr"/>
+      <c r="E382" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="383">
+      <c r="A383" t="inlineStr">
+        <is>
+          <t>40490983</t>
+        </is>
+      </c>
+      <c r="B383" t="inlineStr">
+        <is>
+          <t>Which drug classes were received by individuals in the study before sample sequencing?</t>
+        </is>
+      </c>
+      <c r="C383" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D383" t="inlineStr"/>
+      <c r="E383" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="384">
+      <c r="A384" t="inlineStr">
+        <is>
+          <t>40490983</t>
+        </is>
+      </c>
+      <c r="B384" t="inlineStr">
+        <is>
+          <t>Which drugs were received by individuals in the study before sample sequencing?</t>
+        </is>
+      </c>
+      <c r="C384" t="inlineStr">
+        <is>
+          <t>NRTI, NNRTI, PI</t>
+        </is>
+      </c>
+      <c r="D384" t="inlineStr"/>
+      <c r="E384" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="385">
+      <c r="A385" t="inlineStr">
+        <is>
+          <t>40573423</t>
+        </is>
+      </c>
+      <c r="B385" t="inlineStr">
+        <is>
+          <t>Does the paper report HIV sequences from patient samples?</t>
+        </is>
+      </c>
+      <c r="C385" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D385" t="inlineStr"/>
+      <c r="E385" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="386">
+      <c r="A386" t="inlineStr">
+        <is>
+          <t>40573423</t>
+        </is>
+      </c>
+      <c r="B386" t="inlineStr">
+        <is>
+          <t>From which countries were the sequenced samples obtained?</t>
+        </is>
+      </c>
+      <c r="C386" t="inlineStr">
+        <is>
+          <t>487</t>
+        </is>
+      </c>
+      <c r="D386" t="inlineStr"/>
+      <c r="E386" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="387">
+      <c r="A387" t="inlineStr">
+        <is>
+          <t>40573423</t>
+        </is>
+      </c>
+      <c r="B387" t="inlineStr">
+        <is>
+          <t>From what years were the sequenced samples obtained?</t>
+        </is>
+      </c>
+      <c r="C387" t="inlineStr">
+        <is>
+          <t>South Korea</t>
+        </is>
+      </c>
+      <c r="D387" t="inlineStr"/>
+      <c r="E387" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="388">
+      <c r="A388" t="inlineStr">
+        <is>
+          <t>40573423</t>
+        </is>
+      </c>
+      <c r="B388" t="inlineStr">
+        <is>
+          <t>What method was used for sequencing?</t>
+        </is>
+      </c>
+      <c r="C388" t="inlineStr">
+        <is>
+          <t>2021-2024</t>
+        </is>
+      </c>
+      <c r="D388" t="inlineStr"/>
+      <c r="E388" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="389">
+      <c r="A389" t="inlineStr">
+        <is>
+          <t>40573423</t>
+        </is>
+      </c>
+      <c r="B389" t="inlineStr">
+        <is>
+          <t>What type of samples were sequenced?</t>
+        </is>
+      </c>
+      <c r="C389" t="inlineStr">
+        <is>
+          <t>PR, RT, IN</t>
+        </is>
+      </c>
+      <c r="D389" t="inlineStr"/>
+      <c r="E389" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="390">
+      <c r="A390" t="inlineStr">
+        <is>
+          <t>40596906</t>
+        </is>
+      </c>
+      <c r="B390" t="inlineStr">
+        <is>
+          <t>Does the paper report HIV sequences from patient samples?</t>
+        </is>
+      </c>
+      <c r="C390" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D390" t="inlineStr"/>
+      <c r="E390" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="391">
+      <c r="A391" t="inlineStr">
+        <is>
+          <t>40596906</t>
+        </is>
+      </c>
+      <c r="B391" t="inlineStr">
+        <is>
+          <t>What were the GenBank accession numbers for sequenced HIV isolates?</t>
+        </is>
+      </c>
+      <c r="C391" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D391" t="inlineStr"/>
+      <c r="E391" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="392">
+      <c r="A392" t="inlineStr">
+        <is>
+          <t>40596906</t>
+        </is>
+      </c>
+      <c r="B392" t="inlineStr">
+        <is>
+          <t>Which HIV genes were reported to have been sequenced?</t>
+        </is>
+      </c>
+      <c r="C392" t="inlineStr">
+        <is>
+          <t>PV526713-PV526742</t>
+        </is>
+      </c>
+      <c r="D392" t="inlineStr"/>
+      <c r="E392" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="393">
+      <c r="A393" t="inlineStr">
+        <is>
+          <t>40596906</t>
+        </is>
+      </c>
+      <c r="B393" t="inlineStr">
+        <is>
+          <t>From which countries were the sequenced samples obtained?</t>
+        </is>
+      </c>
+      <c r="C393" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="D393" t="inlineStr"/>
+      <c r="E393" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="394">
+      <c r="A394" t="inlineStr">
+        <is>
+          <t>40596906</t>
+        </is>
+      </c>
+      <c r="B394" t="inlineStr">
+        <is>
+          <t>From what years were the sequenced samples obtained?</t>
+        </is>
+      </c>
+      <c r="C394" t="inlineStr">
+        <is>
+          <t>Brazil</t>
+        </is>
+      </c>
+      <c r="D394" t="inlineStr"/>
+      <c r="E394" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="395">
+      <c r="A395" t="inlineStr">
+        <is>
+          <t>40596906</t>
+        </is>
+      </c>
+      <c r="B395" t="inlineStr">
+        <is>
+          <t>What method was used for sequencing?</t>
+        </is>
+      </c>
+      <c r="C395" t="inlineStr">
+        <is>
+          <t>2007-2022</t>
+        </is>
+      </c>
+      <c r="D395" t="inlineStr"/>
+      <c r="E395" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="396">
+      <c r="A396" t="inlineStr">
+        <is>
+          <t>40596906</t>
+        </is>
+      </c>
+      <c r="B396" t="inlineStr">
+        <is>
+          <t>What type of samples were sequenced?</t>
+        </is>
+      </c>
+      <c r="C396" t="inlineStr">
+        <is>
+          <t>RT, PR</t>
+        </is>
+      </c>
+      <c r="D396" t="inlineStr"/>
+      <c r="E396" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="397">
+      <c r="A397" t="inlineStr">
+        <is>
+          <t>40596906</t>
+        </is>
+      </c>
+      <c r="B397" t="inlineStr">
+        <is>
+          <t>How many individuals had samples obtained for HIV sequencing?</t>
+        </is>
+      </c>
+      <c r="C397" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D397" t="inlineStr"/>
+      <c r="E397" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="398">
+      <c r="A398" t="inlineStr">
+        <is>
+          <t>40596906</t>
+        </is>
+      </c>
+      <c r="B398" t="inlineStr">
+        <is>
+          <t>Which drug classes were received by individuals in the study before sample sequencing?</t>
+        </is>
+      </c>
+      <c r="C398" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D398" t="inlineStr"/>
+      <c r="E398" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="399">
+      <c r="A399" t="inlineStr">
+        <is>
+          <t>40596906</t>
+        </is>
+      </c>
+      <c r="B399" t="inlineStr">
+        <is>
+          <t>Which drugs were received by individuals in the study before sample sequencing?</t>
+        </is>
+      </c>
+      <c r="C399" t="inlineStr">
+        <is>
+          <t>NRTI, NNRTI</t>
+        </is>
+      </c>
+      <c r="D399" t="inlineStr"/>
+      <c r="E399" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="400">
+      <c r="A400" t="inlineStr">
+        <is>
+          <t>40713598</t>
+        </is>
+      </c>
+      <c r="B400" t="inlineStr">
+        <is>
+          <t>Does the paper report HIV sequences from patient samples?</t>
+        </is>
+      </c>
+      <c r="C400" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D400" t="inlineStr"/>
+      <c r="E400" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="401">
+      <c r="A401" t="inlineStr">
+        <is>
+          <t>40713598</t>
+        </is>
+      </c>
+      <c r="B401" t="inlineStr">
+        <is>
+          <t>From which countries were the sequenced samples obtained?</t>
+        </is>
+      </c>
+      <c r="C401" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="D401" t="inlineStr"/>
+      <c r="E401" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="402">
+      <c r="A402" t="inlineStr">
+        <is>
+          <t>40713598</t>
+        </is>
+      </c>
+      <c r="B402" t="inlineStr">
+        <is>
+          <t>From what years were the sequenced samples obtained?</t>
+        </is>
+      </c>
+      <c r="C402" t="inlineStr">
+        <is>
+          <t>Ghana</t>
+        </is>
+      </c>
+      <c r="D402" t="inlineStr"/>
+      <c r="E402" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="403">
+      <c r="A403" t="inlineStr">
+        <is>
+          <t>40713598</t>
+        </is>
+      </c>
+      <c r="B403" t="inlineStr">
+        <is>
+          <t>What type of samples were sequenced?</t>
+        </is>
+      </c>
+      <c r="C403" t="inlineStr">
+        <is>
+          <t>RT</t>
+        </is>
+      </c>
+      <c r="D403" t="inlineStr"/>
+      <c r="E403" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="404">
+      <c r="A404" t="inlineStr">
+        <is>
+          <t>40713598</t>
+        </is>
+      </c>
+      <c r="B404" t="inlineStr">
+        <is>
+          <t>How many individuals had samples obtained for HIV sequencing?</t>
+        </is>
+      </c>
+      <c r="C404" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D404" t="inlineStr"/>
+      <c r="E404" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="405">
+      <c r="A405" t="inlineStr">
+        <is>
+          <t>40713598</t>
+        </is>
+      </c>
+      <c r="B405" t="inlineStr">
+        <is>
+          <t>Which drug classes were received by individuals in the study before sample sequencing?</t>
+        </is>
+      </c>
+      <c r="C405" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D405" t="inlineStr"/>
+      <c r="E405" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="406">
+      <c r="A406" t="inlineStr">
+        <is>
+          <t>40713598</t>
+        </is>
+      </c>
+      <c r="B406" t="inlineStr">
+        <is>
+          <t>Which drugs were received by individuals in the study before sample sequencing?</t>
+        </is>
+      </c>
+      <c r="C406" t="inlineStr">
+        <is>
+          <t>NRTI, NNRTI</t>
+        </is>
+      </c>
+      <c r="D406" t="inlineStr"/>
+      <c r="E406" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="407">
+      <c r="A407" t="inlineStr">
+        <is>
+          <t>40763144</t>
+        </is>
+      </c>
+      <c r="B407" t="inlineStr">
+        <is>
+          <t>Does the paper report HIV sequences from patient samples?</t>
+        </is>
+      </c>
+      <c r="C407" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D407" t="inlineStr"/>
+      <c r="E407" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="408">
+      <c r="A408" t="inlineStr">
+        <is>
+          <t>40763144</t>
+        </is>
+      </c>
+      <c r="B408" t="inlineStr">
+        <is>
+          <t>From which countries were the sequenced samples obtained?</t>
+        </is>
+      </c>
+      <c r="C408" t="inlineStr">
+        <is>
+          <t>295</t>
+        </is>
+      </c>
+      <c r="D408" t="inlineStr"/>
+      <c r="E408" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="409">
+      <c r="A409" t="inlineStr">
+        <is>
+          <t>40763144</t>
+        </is>
+      </c>
+      <c r="B409" t="inlineStr">
+        <is>
+          <t>From what years were the sequenced samples obtained?</t>
+        </is>
+      </c>
+      <c r="C409" t="inlineStr">
+        <is>
+          <t>Uganda</t>
+        </is>
+      </c>
+      <c r="D409" t="inlineStr"/>
+      <c r="E409" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="410">
+      <c r="A410" t="inlineStr">
+        <is>
+          <t>40763144</t>
+        </is>
+      </c>
+      <c r="B410" t="inlineStr">
+        <is>
+          <t>What method was used for sequencing?</t>
+        </is>
+      </c>
+      <c r="C410" t="inlineStr">
+        <is>
+          <t>2021-2023</t>
+        </is>
+      </c>
+      <c r="D410" t="inlineStr"/>
+      <c r="E410" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="411">
+      <c r="A411" t="inlineStr">
+        <is>
+          <t>40763144</t>
+        </is>
+      </c>
+      <c r="B411" t="inlineStr">
+        <is>
+          <t>What type of samples were sequenced?</t>
+        </is>
+      </c>
+      <c r="C411" t="inlineStr">
+        <is>
+          <t>PR, RT, IN</t>
+        </is>
+      </c>
+      <c r="D411" t="inlineStr"/>
+      <c r="E411" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="412">
+      <c r="A412" t="inlineStr">
+        <is>
+          <t>40763144</t>
+        </is>
+      </c>
+      <c r="B412" t="inlineStr">
+        <is>
+          <t>How many individuals had samples obtained for HIV sequencing?</t>
+        </is>
+      </c>
+      <c r="C412" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D412" t="inlineStr"/>
+      <c r="E412" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="413">
+      <c r="A413" t="inlineStr">
+        <is>
+          <t>40763144</t>
+        </is>
+      </c>
+      <c r="B413" t="inlineStr">
+        <is>
+          <t>Which drug classes were received by individuals in the study before sample sequencing?</t>
+        </is>
+      </c>
+      <c r="C413" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D413" t="inlineStr"/>
+      <c r="E413" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="414">
+      <c r="A414" t="inlineStr">
+        <is>
+          <t>40763144</t>
+        </is>
+      </c>
+      <c r="B414" t="inlineStr">
+        <is>
+          <t>Which drugs were received by individuals in the study before sample sequencing?</t>
+        </is>
+      </c>
+      <c r="C414" t="inlineStr">
+        <is>
+          <t>NRTI, NNRTI, PI, INSTI</t>
+        </is>
+      </c>
+      <c r="D414" t="inlineStr"/>
+      <c r="E414" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="415">
+      <c r="A415" t="inlineStr">
+        <is>
+          <t>40779404</t>
+        </is>
+      </c>
+      <c r="B415" t="inlineStr">
+        <is>
+          <t>Does the paper report HIV sequences from patient samples?</t>
+        </is>
+      </c>
+      <c r="C415" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D415" t="inlineStr"/>
+      <c r="E415" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="416">
+      <c r="A416" t="inlineStr">
+        <is>
+          <t>40779404</t>
+        </is>
+      </c>
+      <c r="B416" t="inlineStr">
+        <is>
+          <t>From which countries were the sequenced samples obtained?</t>
+        </is>
+      </c>
+      <c r="C416" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="D416" t="inlineStr"/>
+      <c r="E416" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="417">
+      <c r="A417" t="inlineStr">
+        <is>
+          <t>40779404</t>
+        </is>
+      </c>
+      <c r="B417" t="inlineStr">
+        <is>
+          <t>What type of samples were sequenced?</t>
+        </is>
+      </c>
+      <c r="C417" t="inlineStr">
+        <is>
+          <t>RT,PR,IN</t>
+        </is>
+      </c>
+      <c r="D417" t="inlineStr"/>
+      <c r="E417" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="418">
+      <c r="A418" t="inlineStr">
+        <is>
+          <t>40779404</t>
+        </is>
+      </c>
+      <c r="B418" t="inlineStr">
+        <is>
+          <t>Does the paper report HIV sequences from individuals who had previously received ARV drugs?</t>
+        </is>
+      </c>
+      <c r="C418" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D418" t="inlineStr"/>
+      <c r="E418" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="419">
+      <c r="A419" t="inlineStr">
+        <is>
+          <t>40779404</t>
+        </is>
+      </c>
+      <c r="B419" t="inlineStr">
+        <is>
+          <t>Which drug classes were received by individuals in the study before sample sequencing?</t>
+        </is>
+      </c>
+      <c r="C419" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D419" t="inlineStr"/>
+      <c r="E419" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="420">
+      <c r="A420" t="inlineStr">
+        <is>
+          <t>40779404</t>
+        </is>
+      </c>
+      <c r="B420" t="inlineStr">
+        <is>
+          <t>Which drugs were received by individuals in the study before sample sequencing?</t>
+        </is>
+      </c>
+      <c r="C420" t="inlineStr">
+        <is>
+          <t>NRTI,NNRTI,PI, INSTI</t>
+        </is>
+      </c>
+      <c r="D420" t="inlineStr"/>
+      <c r="E420" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="421">
+      <c r="A421" t="inlineStr">
+        <is>
+          <t>40839365</t>
+        </is>
+      </c>
+      <c r="B421" t="inlineStr">
+        <is>
+          <t>Does the paper report HIV sequences from patient samples?</t>
+        </is>
+      </c>
+      <c r="C421" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D421" t="inlineStr"/>
+      <c r="E421" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="422">
+      <c r="A422" t="inlineStr">
+        <is>
+          <t>40839365</t>
+        </is>
+      </c>
+      <c r="B422" t="inlineStr">
+        <is>
+          <t>From which countries were the sequenced samples obtained?</t>
+        </is>
+      </c>
+      <c r="C422" t="inlineStr">
+        <is>
+          <t>212</t>
+        </is>
+      </c>
+      <c r="D422" t="inlineStr"/>
+      <c r="E422" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="423">
+      <c r="A423" t="inlineStr">
+        <is>
+          <t>40839365</t>
+        </is>
+      </c>
+      <c r="B423" t="inlineStr">
+        <is>
+          <t>From what years were the sequenced samples obtained?</t>
+        </is>
+      </c>
+      <c r="C423" t="inlineStr">
+        <is>
+          <t>Malawi</t>
+        </is>
+      </c>
+      <c r="D423" t="inlineStr"/>
+      <c r="E423" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="424">
+      <c r="A424" t="inlineStr">
+        <is>
+          <t>40839365</t>
+        </is>
+      </c>
+      <c r="B424" t="inlineStr">
+        <is>
+          <t>What method was used for sequencing?</t>
+        </is>
+      </c>
+      <c r="C424" t="inlineStr">
+        <is>
+          <t>2022-2023</t>
+        </is>
+      </c>
+      <c r="D424" t="inlineStr"/>
+      <c r="E424" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="425">
+      <c r="A425" t="inlineStr">
+        <is>
+          <t>40839365</t>
+        </is>
+      </c>
+      <c r="B425" t="inlineStr">
+        <is>
+          <t>What type of samples were sequenced?</t>
+        </is>
+      </c>
+      <c r="C425" t="inlineStr">
+        <is>
+          <t>RT, IN</t>
+        </is>
+      </c>
+      <c r="D425" t="inlineStr"/>
+      <c r="E425" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="426">
+      <c r="A426" t="inlineStr">
+        <is>
+          <t>40839365</t>
+        </is>
+      </c>
+      <c r="B426" t="inlineStr">
+        <is>
+          <t>How many individuals had samples obtained for HIV sequencing?</t>
+        </is>
+      </c>
+      <c r="C426" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D426" t="inlineStr"/>
+      <c r="E426" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="427">
+      <c r="A427" t="inlineStr">
+        <is>
+          <t>40839365</t>
+        </is>
+      </c>
+      <c r="B427" t="inlineStr">
+        <is>
+          <t>Which drug classes were received by individuals in the study before sample sequencing?</t>
+        </is>
+      </c>
+      <c r="C427" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D427" t="inlineStr"/>
+      <c r="E427" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="428">
+      <c r="A428" t="inlineStr">
+        <is>
+          <t>40839365</t>
+        </is>
+      </c>
+      <c r="B428" t="inlineStr">
+        <is>
+          <t>Which drugs were received by individuals in the study before sample sequencing?</t>
+        </is>
+      </c>
+      <c r="C428" t="inlineStr">
+        <is>
+          <t>NRTI, NNRTI, INSTI</t>
+        </is>
+      </c>
+      <c r="D428" t="inlineStr"/>
+      <c r="E428" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="429">
+      <c r="A429" t="inlineStr">
+        <is>
+          <t>40857111</t>
+        </is>
+      </c>
+      <c r="B429" t="inlineStr">
+        <is>
+          <t>Does the paper report HIV sequences from patient samples?</t>
+        </is>
+      </c>
+      <c r="C429" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D429" t="inlineStr"/>
+      <c r="E429" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="430">
+      <c r="A430" t="inlineStr">
+        <is>
+          <t>40857111</t>
+        </is>
+      </c>
+      <c r="B430" t="inlineStr">
+        <is>
+          <t>From which countries were the sequenced samples obtained?</t>
+        </is>
+      </c>
+      <c r="C430" t="inlineStr">
+        <is>
+          <t>7 (Uncertain)</t>
+        </is>
+      </c>
+      <c r="D430" t="inlineStr"/>
+      <c r="E430" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="431">
+      <c r="A431" t="inlineStr">
+        <is>
+          <t>40857111</t>
+        </is>
+      </c>
+      <c r="B431" t="inlineStr">
+        <is>
+          <t>What type of samples were sequenced?</t>
+        </is>
+      </c>
+      <c r="C431" t="inlineStr">
+        <is>
+          <t>RT,PR,IN</t>
+        </is>
+      </c>
+      <c r="D431" t="inlineStr"/>
+      <c r="E431" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="432">
+      <c r="A432" t="inlineStr">
+        <is>
+          <t>40857111</t>
+        </is>
+      </c>
+      <c r="B432" t="inlineStr">
+        <is>
+          <t>How many individuals had samples obtained for HIV sequencing?</t>
+        </is>
+      </c>
+      <c r="C432" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D432" t="inlineStr"/>
+      <c r="E432" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="433">
+      <c r="A433" t="inlineStr">
+        <is>
+          <t>40857111</t>
+        </is>
+      </c>
+      <c r="B433" t="inlineStr">
+        <is>
+          <t>Does the paper report HIV sequences from individuals who had previously received ARV drugs?</t>
+        </is>
+      </c>
+      <c r="C433" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D433" t="inlineStr"/>
+      <c r="E433" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="434">
+      <c r="A434" t="inlineStr">
+        <is>
+          <t>40857111</t>
+        </is>
+      </c>
+      <c r="B434" t="inlineStr">
+        <is>
+          <t>Which drug classes were received by individuals in the study before sample sequencing?</t>
+        </is>
+      </c>
+      <c r="C434" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D434" t="inlineStr"/>
+      <c r="E434" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="435">
+      <c r="A435" t="inlineStr">
+        <is>
+          <t>40857111</t>
+        </is>
+      </c>
+      <c r="B435" t="inlineStr">
+        <is>
+          <t>Which drugs were received by individuals in the study before sample sequencing?</t>
+        </is>
+      </c>
+      <c r="C435" t="inlineStr">
+        <is>
+          <t>NRTI, INSTI</t>
+        </is>
+      </c>
+      <c r="D435" t="inlineStr"/>
+      <c r="E435" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="436">
+      <c r="A436" t="inlineStr">
+        <is>
+          <t>40872801</t>
+        </is>
+      </c>
+      <c r="B436" t="inlineStr">
+        <is>
+          <t>From what years were the sequenced samples obtained?</t>
+        </is>
+      </c>
+      <c r="C436" t="inlineStr">
+        <is>
+          <t>Tanzania</t>
+        </is>
+      </c>
+      <c r="D436" t="inlineStr"/>
+      <c r="E436" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="437">
+      <c r="A437" t="inlineStr">
+        <is>
+          <t>40872801</t>
+        </is>
+      </c>
+      <c r="B437" t="inlineStr">
+        <is>
+          <t>What method was used for sequencing?</t>
+        </is>
+      </c>
+      <c r="C437" t="inlineStr">
+        <is>
+          <t>2004-2021</t>
+        </is>
+      </c>
+      <c r="D437" t="inlineStr"/>
+      <c r="E437" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="438">
+      <c r="A438" t="inlineStr">
+        <is>
+          <t>40872801</t>
+        </is>
+      </c>
+      <c r="B438" t="inlineStr">
+        <is>
+          <t>What type of samples were sequenced?</t>
+        </is>
+      </c>
+      <c r="C438" t="inlineStr">
+        <is>
+          <t>RT, PR</t>
+        </is>
+      </c>
+      <c r="D438" t="inlineStr"/>
+      <c r="E438" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="439">
+      <c r="A439" t="inlineStr">
+        <is>
+          <t>40872801</t>
+        </is>
+      </c>
+      <c r="B439" t="inlineStr">
+        <is>
+          <t>How many individuals had samples obtained for HIV sequencing?</t>
+        </is>
+      </c>
+      <c r="C439" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D439" t="inlineStr"/>
+      <c r="E439" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="440">
+      <c r="A440" t="inlineStr">
+        <is>
+          <t>40872801</t>
+        </is>
+      </c>
+      <c r="B440" t="inlineStr">
+        <is>
+          <t>Which drug classes were received by individuals in the study before sample sequencing?</t>
+        </is>
+      </c>
+      <c r="C440" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D440" t="inlineStr"/>
+      <c r="E440" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="441">
+      <c r="A441" t="inlineStr">
+        <is>
+          <t>40872801</t>
+        </is>
+      </c>
+      <c r="B441" t="inlineStr">
+        <is>
+          <t>Which drugs were received by individuals in the study before sample sequencing?</t>
+        </is>
+      </c>
+      <c r="C441" t="inlineStr">
+        <is>
+          <t>NRTI, NNRTI, PI</t>
+        </is>
+      </c>
+      <c r="D441" t="inlineStr"/>
+      <c r="E441" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="442">
+      <c r="A442" t="inlineStr">
+        <is>
+          <t>40938120</t>
+        </is>
+      </c>
+      <c r="B442" t="inlineStr">
+        <is>
+          <t>Does the paper report HIV sequences from patient samples?</t>
+        </is>
+      </c>
+      <c r="C442" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D442" t="inlineStr"/>
+      <c r="E442" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="443">
+      <c r="A443" t="inlineStr">
+        <is>
+          <t>40938120</t>
+        </is>
+      </c>
+      <c r="B443" t="inlineStr">
+        <is>
+          <t>What were the GenBank accession numbers for sequenced HIV isolates?</t>
+        </is>
+      </c>
+      <c r="C443" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D443" t="inlineStr"/>
+      <c r="E443" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="444">
+      <c r="A444" t="inlineStr">
+        <is>
+          <t>40938120</t>
+        </is>
+      </c>
+      <c r="B444" t="inlineStr">
+        <is>
+          <t>Which HIV genes were reported to have been sequenced?</t>
+        </is>
+      </c>
+      <c r="C444" t="inlineStr">
+        <is>
+          <t>PX133190–PX134237</t>
+        </is>
+      </c>
+      <c r="D444" t="inlineStr"/>
+      <c r="E444" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="445">
+      <c r="A445" t="inlineStr">
+        <is>
+          <t>40938120</t>
+        </is>
+      </c>
+      <c r="B445" t="inlineStr">
+        <is>
+          <t>From which countries were the sequenced samples obtained?</t>
+        </is>
+      </c>
+      <c r="C445" t="inlineStr">
+        <is>
+          <t>1048</t>
+        </is>
+      </c>
+      <c r="D445" t="inlineStr"/>
+      <c r="E445" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="446">
+      <c r="A446" t="inlineStr">
+        <is>
+          <t>40938120</t>
+        </is>
+      </c>
+      <c r="B446" t="inlineStr">
+        <is>
+          <t>From what years were the sequenced samples obtained?</t>
+        </is>
+      </c>
+      <c r="C446" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="D446" t="inlineStr"/>
+      <c r="E446" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="447">
+      <c r="A447" t="inlineStr">
+        <is>
+          <t>40938120</t>
+        </is>
+      </c>
+      <c r="B447" t="inlineStr">
+        <is>
+          <t>What method was used for sequencing?</t>
+        </is>
+      </c>
+      <c r="C447" t="inlineStr">
+        <is>
+          <t>2019-2022</t>
+        </is>
+      </c>
+      <c r="D447" t="inlineStr"/>
+      <c r="E447" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="448">
+      <c r="A448" t="inlineStr">
+        <is>
+          <t>40938120</t>
+        </is>
+      </c>
+      <c r="B448" t="inlineStr">
+        <is>
+          <t>What type of samples were sequenced?</t>
+        </is>
+      </c>
+      <c r="C448" t="inlineStr">
+        <is>
+          <t>RT, PR</t>
+        </is>
+      </c>
+      <c r="D448" t="inlineStr"/>
+      <c r="E448" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="449">
+      <c r="A449" t="inlineStr">
+        <is>
+          <t>40938996</t>
+        </is>
+      </c>
+      <c r="B449" t="inlineStr">
+        <is>
+          <t>Does the paper report in vitro drug susceptibility data?</t>
+        </is>
+      </c>
+      <c r="C449" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D449" t="inlineStr"/>
+      <c r="E449" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="450">
+      <c r="A450" t="inlineStr">
+        <is>
+          <t>40938996</t>
+        </is>
+      </c>
+      <c r="B450" t="inlineStr">
+        <is>
+          <t>Were samples cloned prior to sequencing?</t>
+        </is>
+      </c>
+      <c r="C450" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D450" t="inlineStr"/>
+      <c r="E450" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="451">
+      <c r="A451" t="inlineStr">
+        <is>
+          <t>40938996</t>
+        </is>
+      </c>
+      <c r="B451" t="inlineStr">
+        <is>
+          <t>What type of samples were sequenced?</t>
+        </is>
+      </c>
+      <c r="C451" t="inlineStr">
+        <is>
+          <t>RT, IN, NC, Env</t>
+        </is>
+      </c>
+      <c r="D451" t="inlineStr"/>
+      <c r="E451" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="452">
+      <c r="A452" t="inlineStr">
+        <is>
+          <t>40965168</t>
+        </is>
+      </c>
+      <c r="B452" t="inlineStr">
+        <is>
+          <t>Does the paper report in vitro drug susceptibility data?</t>
+        </is>
+      </c>
+      <c r="C452" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D452" t="inlineStr"/>
+      <c r="E452" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="453">
+      <c r="A453" t="inlineStr">
+        <is>
+          <t>40965168</t>
+        </is>
+      </c>
+      <c r="B453" t="inlineStr">
+        <is>
+          <t>Were samples cloned prior to sequencing?</t>
+        </is>
+      </c>
+      <c r="C453" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D453" t="inlineStr"/>
+      <c r="E453" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="454">
+      <c r="A454" t="inlineStr">
+        <is>
+          <t>40965168</t>
+        </is>
+      </c>
+      <c r="B454" t="inlineStr">
+        <is>
+          <t>What type of samples were sequenced?</t>
+        </is>
+      </c>
+      <c r="C454" t="inlineStr">
+        <is>
+          <t>CA</t>
+        </is>
+      </c>
+      <c r="D454" t="inlineStr"/>
+      <c r="E454" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="455">
+      <c r="A455" t="inlineStr">
+        <is>
+          <t>40974886</t>
+        </is>
+      </c>
+      <c r="B455" t="inlineStr">
+        <is>
+          <t>Does the paper report HIV sequences from patient samples?</t>
+        </is>
+      </c>
+      <c r="C455" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D455" t="inlineStr"/>
+      <c r="E455" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="456">
+      <c r="A456" t="inlineStr">
+        <is>
+          <t>40974886</t>
+        </is>
+      </c>
+      <c r="B456" t="inlineStr">
+        <is>
+          <t>From which countries were the sequenced samples obtained?</t>
+        </is>
+      </c>
+      <c r="C456" t="inlineStr">
+        <is>
+          <t>223</t>
+        </is>
+      </c>
+      <c r="D456" t="inlineStr"/>
+      <c r="E456" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="457">
+      <c r="A457" t="inlineStr">
+        <is>
+          <t>40974886</t>
+        </is>
+      </c>
+      <c r="B457" t="inlineStr">
+        <is>
+          <t>What method was used for sequencing?</t>
+        </is>
+      </c>
+      <c r="C457" t="inlineStr">
+        <is>
+          <t>1997-2019</t>
+        </is>
+      </c>
+      <c r="D457" t="inlineStr"/>
+      <c r="E457" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="458">
+      <c r="A458" t="inlineStr">
+        <is>
+          <t>40974886</t>
+        </is>
+      </c>
+      <c r="B458" t="inlineStr">
+        <is>
+          <t>What type of samples were sequenced?</t>
+        </is>
+      </c>
+      <c r="C458" t="inlineStr">
+        <is>
+          <t>RT,PR,IN</t>
+        </is>
+      </c>
+      <c r="D458" t="inlineStr"/>
+      <c r="E458" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="459">
+      <c r="A459" t="inlineStr">
+        <is>
+          <t>40974886</t>
+        </is>
+      </c>
+      <c r="B459" t="inlineStr">
+        <is>
+          <t>How many individuals had samples obtained for HIV sequencing?</t>
+        </is>
+      </c>
+      <c r="C459" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D459" t="inlineStr"/>
+      <c r="E459" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="460">
+      <c r="A460" t="inlineStr">
+        <is>
+          <t>40974886</t>
+        </is>
+      </c>
+      <c r="B460" t="inlineStr">
+        <is>
+          <t>Does the paper report HIV sequences from individuals who had previously received ARV drugs?</t>
+        </is>
+      </c>
+      <c r="C460" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D460" t="inlineStr"/>
+      <c r="E460" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="461">
+      <c r="A461" t="inlineStr">
+        <is>
+          <t>40974886</t>
+        </is>
+      </c>
+      <c r="B461" t="inlineStr">
+        <is>
+          <t>Which drug classes were received by individuals in the study before sample sequencing?</t>
+        </is>
+      </c>
+      <c r="C461" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D461" t="inlineStr"/>
+      <c r="E461" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="462">
+      <c r="A462" t="inlineStr">
+        <is>
+          <t>40974886</t>
+        </is>
+      </c>
+      <c r="B462" t="inlineStr">
+        <is>
+          <t>Which drugs were received by individuals in the study before sample sequencing?</t>
+        </is>
+      </c>
+      <c r="C462" t="inlineStr">
+        <is>
+          <t>NRTI, NNRTI, PI, INSTI</t>
+        </is>
+      </c>
+      <c r="D462" t="inlineStr"/>
+      <c r="E462" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="463">
+      <c r="A463" t="inlineStr">
+        <is>
+          <t>41004608</t>
+        </is>
+      </c>
+      <c r="B463" t="inlineStr">
+        <is>
+          <t>Does the paper report HIV sequences from patient samples?</t>
+        </is>
+      </c>
+      <c r="C463" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D463" t="inlineStr"/>
+      <c r="E463" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="464">
+      <c r="A464" t="inlineStr">
+        <is>
+          <t>41004608</t>
+        </is>
+      </c>
+      <c r="B464" t="inlineStr">
+        <is>
+          <t>From which countries were the sequenced samples obtained?</t>
+        </is>
+      </c>
+      <c r="C464" t="inlineStr">
+        <is>
+          <t>1182</t>
+        </is>
+      </c>
+      <c r="D464" t="inlineStr"/>
+      <c r="E464" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="465">
+      <c r="A465" t="inlineStr">
+        <is>
+          <t>41004608</t>
+        </is>
+      </c>
+      <c r="B465" t="inlineStr">
+        <is>
+          <t>From what years were the sequenced samples obtained?</t>
+        </is>
+      </c>
+      <c r="C465" t="inlineStr">
+        <is>
+          <t>UK</t>
+        </is>
+      </c>
+      <c r="D465" t="inlineStr"/>
+      <c r="E465" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="466">
+      <c r="A466" t="inlineStr">
+        <is>
+          <t>41004608</t>
+        </is>
+      </c>
+      <c r="B466" t="inlineStr">
+        <is>
+          <t>What method was used for sequencing?</t>
+        </is>
+      </c>
+      <c r="C466" t="inlineStr">
+        <is>
+          <t>2015-2021</t>
+        </is>
+      </c>
+      <c r="D466" t="inlineStr"/>
+      <c r="E466" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="467">
+      <c r="A467" t="inlineStr">
+        <is>
+          <t>41004608</t>
+        </is>
+      </c>
+      <c r="B467" t="inlineStr">
+        <is>
+          <t>What type of samples were sequenced?</t>
+        </is>
+      </c>
+      <c r="C467" t="inlineStr">
+        <is>
+          <t>Whole genome</t>
+        </is>
+      </c>
+      <c r="D467" t="inlineStr"/>
+      <c r="E467" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="468">
+      <c r="A468" t="inlineStr">
+        <is>
+          <t>41012586</t>
+        </is>
+      </c>
+      <c r="B468" t="inlineStr">
+        <is>
+          <t>Does the paper report HIV sequences from patient samples?</t>
+        </is>
+      </c>
+      <c r="C468" t="inlineStr">
+        <is>
+          <t>Yes (Only past sequences)</t>
+        </is>
+      </c>
+      <c r="D468" t="inlineStr"/>
+      <c r="E468" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="469">
+      <c r="A469" t="inlineStr">
+        <is>
+          <t>41012586</t>
+        </is>
+      </c>
+      <c r="B469" t="inlineStr">
+        <is>
+          <t>From which countries were the sequenced samples obtained?</t>
+        </is>
+      </c>
+      <c r="C469" t="inlineStr">
+        <is>
+          <t>249 (uncertain)</t>
+        </is>
+      </c>
+      <c r="D469" t="inlineStr"/>
+      <c r="E469" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="470">
+      <c r="A470" t="inlineStr">
+        <is>
+          <t>41012586</t>
+        </is>
+      </c>
+      <c r="B470" t="inlineStr">
+        <is>
+          <t>From what years were the sequenced samples obtained?</t>
+        </is>
+      </c>
+      <c r="C470" t="inlineStr">
+        <is>
+          <t>Italy</t>
+        </is>
+      </c>
+      <c r="D470" t="inlineStr"/>
+      <c r="E470" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="471">
+      <c r="A471" t="inlineStr">
+        <is>
+          <t>41012586</t>
+        </is>
+      </c>
+      <c r="B471" t="inlineStr">
+        <is>
+          <t>What type of samples were sequenced?</t>
+        </is>
+      </c>
+      <c r="C471" t="inlineStr">
+        <is>
+          <t>PR, RT, IN (presumably)</t>
+        </is>
+      </c>
+      <c r="D471" t="inlineStr"/>
+      <c r="E471" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="472">
+      <c r="A472" t="inlineStr">
+        <is>
+          <t>41012586</t>
+        </is>
+      </c>
+      <c r="B472" t="inlineStr">
+        <is>
+          <t>How many individuals had samples obtained for HIV sequencing?</t>
+        </is>
+      </c>
+      <c r="C472" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D472" t="inlineStr"/>
+      <c r="E472" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="473">
+      <c r="A473" t="inlineStr">
+        <is>
+          <t>41012586</t>
+        </is>
+      </c>
+      <c r="B473" t="inlineStr">
+        <is>
+          <t>Which drug classes were received by individuals in the study before sample sequencing?</t>
+        </is>
+      </c>
+      <c r="C473" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D473" t="inlineStr"/>
+      <c r="E473" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="474">
+      <c r="A474" t="inlineStr">
+        <is>
+          <t>41012586</t>
+        </is>
+      </c>
+      <c r="B474" t="inlineStr">
+        <is>
+          <t>Which drugs were received by individuals in the study before sample sequencing?</t>
+        </is>
+      </c>
+      <c r="C474" t="inlineStr">
+        <is>
+          <t>PI, INSTI, NRTI (presumably)</t>
+        </is>
+      </c>
+      <c r="D474" t="inlineStr"/>
+      <c r="E474" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="475">
+      <c r="A475" t="inlineStr">
+        <is>
+          <t>41023944</t>
+        </is>
+      </c>
+      <c r="B475" t="inlineStr">
+        <is>
+          <t>Does the paper report HIV sequences from patient samples?</t>
+        </is>
+      </c>
+      <c r="C475" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D475" t="inlineStr"/>
+      <c r="E475" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="476">
+      <c r="A476" t="inlineStr">
+        <is>
+          <t>41023944</t>
+        </is>
+      </c>
+      <c r="B476" t="inlineStr">
+        <is>
+          <t>From which countries were the sequenced samples obtained?</t>
+        </is>
+      </c>
+      <c r="C476" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+      <c r="D476" t="inlineStr"/>
+      <c r="E476" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="477">
+      <c r="A477" t="inlineStr">
+        <is>
+          <t>41023944</t>
+        </is>
+      </c>
+      <c r="B477" t="inlineStr">
+        <is>
+          <t>From what years were the sequenced samples obtained?</t>
+        </is>
+      </c>
+      <c r="C477" t="inlineStr">
+        <is>
+          <t>Mozambique</t>
+        </is>
+      </c>
+      <c r="D477" t="inlineStr"/>
+      <c r="E477" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="478">
+      <c r="A478" t="inlineStr">
+        <is>
+          <t>41023944</t>
+        </is>
+      </c>
+      <c r="B478" t="inlineStr">
+        <is>
+          <t>What method was used for sequencing?</t>
+        </is>
+      </c>
+      <c r="C478" t="inlineStr">
+        <is>
+          <t>2022-2024</t>
+        </is>
+      </c>
+      <c r="D478" t="inlineStr"/>
+      <c r="E478" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="479">
+      <c r="A479" t="inlineStr">
+        <is>
+          <t>41023944</t>
+        </is>
+      </c>
+      <c r="B479" t="inlineStr">
+        <is>
+          <t>What type of samples were sequenced?</t>
+        </is>
+      </c>
+      <c r="C479" t="inlineStr">
+        <is>
+          <t>RT,IN</t>
+        </is>
+      </c>
+      <c r="D479" t="inlineStr"/>
+      <c r="E479" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="480">
+      <c r="A480" t="inlineStr">
+        <is>
+          <t>41023944</t>
+        </is>
+      </c>
+      <c r="B480" t="inlineStr">
+        <is>
+          <t>How many individuals had samples obtained for HIV sequencing?</t>
+        </is>
+      </c>
+      <c r="C480" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D480" t="inlineStr"/>
+      <c r="E480" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="481">
+      <c r="A481" t="inlineStr">
+        <is>
+          <t>41023944</t>
+        </is>
+      </c>
+      <c r="B481" t="inlineStr">
+        <is>
+          <t>Which drug classes were received by individuals in the study before sample sequencing?</t>
+        </is>
+      </c>
+      <c r="C481" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D481" t="inlineStr"/>
+      <c r="E481" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="482">
+      <c r="A482" t="inlineStr">
+        <is>
+          <t>41023944</t>
+        </is>
+      </c>
+      <c r="B482" t="inlineStr">
+        <is>
+          <t>Which drugs were received by individuals in the study before sample sequencing?</t>
+        </is>
+      </c>
+      <c r="C482" t="inlineStr">
+        <is>
+          <t>NRTI,NNRTI,INSTI</t>
+        </is>
+      </c>
+      <c r="D482" t="inlineStr"/>
+      <c r="E482" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="483">
+      <c r="A483" t="inlineStr">
+        <is>
+          <t>41029850</t>
+        </is>
+      </c>
+      <c r="B483" t="inlineStr">
+        <is>
+          <t>Does the paper report HIV sequences from patient samples?</t>
+        </is>
+      </c>
+      <c r="C483" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D483" t="inlineStr"/>
+      <c r="E483" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="484">
+      <c r="A484" t="inlineStr">
+        <is>
+          <t>41029850</t>
+        </is>
+      </c>
+      <c r="B484" t="inlineStr">
+        <is>
+          <t>What were the GenBank accession numbers for sequenced HIV isolates?</t>
+        </is>
+      </c>
+      <c r="C484" t="inlineStr">
+        <is>
+          <t>Yes (some)</t>
+        </is>
+      </c>
+      <c r="D484" t="inlineStr"/>
+      <c r="E484" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="485">
+      <c r="A485" t="inlineStr">
+        <is>
+          <t>41029850</t>
+        </is>
+      </c>
+      <c r="B485" t="inlineStr">
+        <is>
+          <t>Which HIV genes were reported to have been sequenced?</t>
+        </is>
+      </c>
+      <c r="C485" t="inlineStr">
+        <is>
+          <t>PQ893197, PQ893192, OQ985810, OR259747 and PQ893191 &amp; submission ID: 2961867)</t>
+        </is>
+      </c>
+      <c r="D485" t="inlineStr"/>
+      <c r="E485" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="486">
+      <c r="A486" t="inlineStr">
+        <is>
+          <t>41029850</t>
+        </is>
+      </c>
+      <c r="B486" t="inlineStr">
+        <is>
+          <t>From which countries were the sequenced samples obtained?</t>
+        </is>
+      </c>
+      <c r="C486" t="inlineStr">
+        <is>
+          <t>203</t>
+        </is>
+      </c>
+      <c r="D486" t="inlineStr"/>
+      <c r="E486" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="487">
+      <c r="A487" t="inlineStr">
+        <is>
+          <t>41029850</t>
+        </is>
+      </c>
+      <c r="B487" t="inlineStr">
+        <is>
+          <t>From what years were the sequenced samples obtained?</t>
+        </is>
+      </c>
+      <c r="C487" t="inlineStr">
+        <is>
+          <t>Cameroon</t>
+        </is>
+      </c>
+      <c r="D487" t="inlineStr"/>
+      <c r="E487" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="488">
+      <c r="A488" t="inlineStr">
+        <is>
+          <t>41029850</t>
+        </is>
+      </c>
+      <c r="B488" t="inlineStr">
+        <is>
+          <t>What method was used for sequencing?</t>
+        </is>
+      </c>
+      <c r="C488" t="inlineStr">
+        <is>
+          <t>2022-2023</t>
+        </is>
+      </c>
+      <c r="D488" t="inlineStr"/>
+      <c r="E488" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="489">
+      <c r="A489" t="inlineStr">
+        <is>
+          <t>41029850</t>
+        </is>
+      </c>
+      <c r="B489" t="inlineStr">
+        <is>
+          <t>What type of samples were sequenced?</t>
+        </is>
+      </c>
+      <c r="C489" t="inlineStr">
+        <is>
+          <t>RT, PR</t>
+        </is>
+      </c>
+      <c r="D489" t="inlineStr"/>
+      <c r="E489" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="490">
+      <c r="A490" t="inlineStr">
+        <is>
+          <t>41029850</t>
+        </is>
+      </c>
+      <c r="B490" t="inlineStr">
+        <is>
+          <t>How many individuals had samples obtained for HIV sequencing?</t>
+        </is>
+      </c>
+      <c r="C490" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D490" t="inlineStr"/>
+      <c r="E490" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="491">
+      <c r="A491" t="inlineStr">
+        <is>
+          <t>41029850</t>
+        </is>
+      </c>
+      <c r="B491" t="inlineStr">
+        <is>
+          <t>Which drug classes were received by individuals in the study before sample sequencing?</t>
+        </is>
+      </c>
+      <c r="C491" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D491" t="inlineStr"/>
+      <c r="E491" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="492">
+      <c r="A492" t="inlineStr">
+        <is>
+          <t>41029850</t>
+        </is>
+      </c>
+      <c r="B492" t="inlineStr">
+        <is>
+          <t>Which drugs were received by individuals in the study before sample sequencing?</t>
+        </is>
+      </c>
+      <c r="C492" t="inlineStr">
+        <is>
+          <t>NRTI, NNRTI, PI, INSTI</t>
+        </is>
+      </c>
+      <c r="D492" t="inlineStr"/>
+      <c r="E492" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="493">
+      <c r="A493" t="inlineStr">
+        <is>
+          <t>41056006</t>
+        </is>
+      </c>
+      <c r="B493" t="inlineStr">
+        <is>
+          <t>Does the paper report HIV sequences from patient samples?</t>
+        </is>
+      </c>
+      <c r="C493" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D493" t="inlineStr"/>
+      <c r="E493" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="494">
+      <c r="A494" t="inlineStr">
+        <is>
+          <t>41056006</t>
+        </is>
+      </c>
+      <c r="B494" t="inlineStr">
+        <is>
+          <t>From which countries were the sequenced samples obtained?</t>
+        </is>
+      </c>
+      <c r="C494" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="D494" t="inlineStr"/>
+      <c r="E494" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="495">
+      <c r="A495" t="inlineStr">
+        <is>
+          <t>41056006</t>
+        </is>
+      </c>
+      <c r="B495" t="inlineStr">
+        <is>
+          <t>What type of samples were sequenced?</t>
+        </is>
+      </c>
+      <c r="C495" t="inlineStr">
+        <is>
+          <t>CA</t>
+        </is>
+      </c>
+      <c r="D495" t="inlineStr"/>
+      <c r="E495" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="496">
+      <c r="A496" t="inlineStr">
+        <is>
+          <t>41056006</t>
+        </is>
+      </c>
+      <c r="B496" t="inlineStr">
+        <is>
+          <t>How many individuals had samples obtained for HIV sequencing?</t>
+        </is>
+      </c>
+      <c r="C496" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D496" t="inlineStr"/>
+      <c r="E496" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="497">
+      <c r="A497" t="inlineStr">
+        <is>
+          <t>41056006</t>
+        </is>
+      </c>
+      <c r="B497" t="inlineStr">
+        <is>
+          <t>Does the paper report HIV sequences from individuals who had previously received ARV drugs?</t>
+        </is>
+      </c>
+      <c r="C497" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D497" t="inlineStr"/>
+      <c r="E497" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="498">
+      <c r="A498" t="inlineStr">
+        <is>
+          <t>41056006</t>
+        </is>
+      </c>
+      <c r="B498" t="inlineStr">
+        <is>
+          <t>Which drug classes were received by individuals in the study before sample sequencing?</t>
+        </is>
+      </c>
+      <c r="C498" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D498" t="inlineStr"/>
+      <c r="E498" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="499">
+      <c r="A499" t="inlineStr">
+        <is>
+          <t>41056006</t>
+        </is>
+      </c>
+      <c r="B499" t="inlineStr">
+        <is>
+          <t>Which drugs were received by individuals in the study before sample sequencing?</t>
+        </is>
+      </c>
+      <c r="C499" t="inlineStr">
+        <is>
+          <t>NRTI, INSTI, CAI</t>
+        </is>
+      </c>
+      <c r="D499" t="inlineStr"/>
+      <c r="E499" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="500">
+      <c r="A500" t="inlineStr">
+        <is>
+          <t>41057785</t>
+        </is>
+      </c>
+      <c r="B500" t="inlineStr">
+        <is>
+          <t>Does the paper report HIV sequences from patient samples?</t>
+        </is>
+      </c>
+      <c r="C500" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D500" t="inlineStr"/>
+      <c r="E500" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="501">
+      <c r="A501" t="inlineStr">
+        <is>
+          <t>41057785</t>
+        </is>
+      </c>
+      <c r="B501" t="inlineStr">
+        <is>
+          <t>From which countries were the sequenced samples obtained?</t>
+        </is>
+      </c>
+      <c r="C501" t="inlineStr">
+        <is>
+          <t>235</t>
+        </is>
+      </c>
+      <c r="D501" t="inlineStr"/>
+      <c r="E501" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="502">
+      <c r="A502" t="inlineStr">
+        <is>
+          <t>41057785</t>
+        </is>
+      </c>
+      <c r="B502" t="inlineStr">
+        <is>
+          <t>From what years were the sequenced samples obtained?</t>
+        </is>
+      </c>
+      <c r="C502" t="inlineStr">
+        <is>
+          <t>Uganda</t>
+        </is>
+      </c>
+      <c r="D502" t="inlineStr"/>
+      <c r="E502" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="503">
+      <c r="A503" t="inlineStr">
+        <is>
+          <t>41057785</t>
+        </is>
+      </c>
+      <c r="B503" t="inlineStr">
+        <is>
+          <t>What method was used for sequencing?</t>
+        </is>
+      </c>
+      <c r="C503" t="inlineStr">
+        <is>
+          <t>2018-2023</t>
+        </is>
+      </c>
+      <c r="D503" t="inlineStr"/>
+      <c r="E503" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="504">
+      <c r="A504" t="inlineStr">
+        <is>
+          <t>41057785</t>
+        </is>
+      </c>
+      <c r="B504" t="inlineStr">
+        <is>
+          <t>What type of samples were sequenced?</t>
+        </is>
+      </c>
+      <c r="C504" t="inlineStr">
+        <is>
+          <t>RT,PR,IN</t>
+        </is>
+      </c>
+      <c r="D504" t="inlineStr"/>
+      <c r="E504" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="505">
+      <c r="A505" t="inlineStr">
+        <is>
+          <t>41057785</t>
+        </is>
+      </c>
+      <c r="B505" t="inlineStr">
+        <is>
+          <t>How many individuals had samples obtained for HIV sequencing?</t>
+        </is>
+      </c>
+      <c r="C505" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D505" t="inlineStr"/>
+      <c r="E505" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="506">
+      <c r="A506" t="inlineStr">
+        <is>
+          <t>41057785</t>
+        </is>
+      </c>
+      <c r="B506" t="inlineStr">
+        <is>
+          <t>Which drug classes were received by individuals in the study before sample sequencing?</t>
+        </is>
+      </c>
+      <c r="C506" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D506" t="inlineStr"/>
+      <c r="E506" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="507">
+      <c r="A507" t="inlineStr">
+        <is>
+          <t>41057785</t>
+        </is>
+      </c>
+      <c r="B507" t="inlineStr">
+        <is>
+          <t>Which drugs were received by individuals in the study before sample sequencing?</t>
+        </is>
+      </c>
+      <c r="C507" t="inlineStr">
+        <is>
+          <t>NRTI,NNRTI,PI, INSTI</t>
+        </is>
+      </c>
+      <c r="D507" t="inlineStr"/>
+      <c r="E507" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="508">
+      <c r="A508" t="inlineStr">
+        <is>
+          <t>41088231</t>
+        </is>
+      </c>
+      <c r="B508" t="inlineStr">
+        <is>
+          <t>Does the paper report HIV sequences from patient samples?</t>
+        </is>
+      </c>
+      <c r="C508" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D508" t="inlineStr"/>
+      <c r="E508" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="509">
+      <c r="A509" t="inlineStr">
+        <is>
+          <t>41088231</t>
+        </is>
+      </c>
+      <c r="B509" t="inlineStr">
+        <is>
+          <t>What were the GenBank accession numbers for sequenced HIV isolates?</t>
+        </is>
+      </c>
+      <c r="C509" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D509" t="inlineStr"/>
+      <c r="E509" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="510">
+      <c r="A510" t="inlineStr">
+        <is>
+          <t>41088231</t>
+        </is>
+      </c>
+      <c r="B510" t="inlineStr">
+        <is>
+          <t>Which HIV genes were reported to have been sequenced?</t>
+        </is>
+      </c>
+      <c r="C510" t="inlineStr">
+        <is>
+          <t>PV187006</t>
+        </is>
+      </c>
+      <c r="D510" t="inlineStr"/>
+      <c r="E510" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="511">
+      <c r="A511" t="inlineStr">
+        <is>
+          <t>41088231</t>
+        </is>
+      </c>
+      <c r="B511" t="inlineStr">
+        <is>
+          <t>From which countries were the sequenced samples obtained?</t>
+        </is>
+      </c>
+      <c r="C511" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D511" t="inlineStr"/>
+      <c r="E511" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="512">
+      <c r="A512" t="inlineStr">
+        <is>
+          <t>41088231</t>
+        </is>
+      </c>
+      <c r="B512" t="inlineStr">
+        <is>
+          <t>From what years were the sequenced samples obtained?</t>
+        </is>
+      </c>
+      <c r="C512" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="D512" t="inlineStr"/>
+      <c r="E512" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="513">
+      <c r="A513" t="inlineStr">
+        <is>
+          <t>41088231</t>
+        </is>
+      </c>
+      <c r="B513" t="inlineStr">
+        <is>
+          <t>What method was used for sequencing?</t>
+        </is>
+      </c>
+      <c r="C513" t="inlineStr">
+        <is>
+          <t>2023</t>
+        </is>
+      </c>
+      <c r="D513" t="inlineStr"/>
+      <c r="E513" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="514">
+      <c r="A514" t="inlineStr">
+        <is>
+          <t>41088231</t>
+        </is>
+      </c>
+      <c r="B514" t="inlineStr">
+        <is>
+          <t>Were samples cloned prior to sequencing?</t>
+        </is>
+      </c>
+      <c r="C514" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D514" t="inlineStr"/>
+      <c r="E514" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="515">
+      <c r="A515" t="inlineStr">
+        <is>
+          <t>41088231</t>
+        </is>
+      </c>
+      <c r="B515" t="inlineStr">
+        <is>
+          <t>What type of samples were sequenced?</t>
+        </is>
+      </c>
+      <c r="C515" t="inlineStr">
+        <is>
+          <t>Whole genome</t>
+        </is>
+      </c>
+      <c r="D515" t="inlineStr"/>
+      <c r="E515" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="516">
+      <c r="A516" t="inlineStr">
+        <is>
+          <t>41091504</t>
+        </is>
+      </c>
+      <c r="B516" t="inlineStr">
+        <is>
+          <t>Were samples cloned prior to sequencing?</t>
+        </is>
+      </c>
+      <c r="C516" t="inlineStr">
+        <is>
+          <t>Yes (site-directed mutants)</t>
+        </is>
+      </c>
+      <c r="D516" t="inlineStr"/>
+      <c r="E516" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="517">
+      <c r="A517" t="inlineStr">
+        <is>
+          <t>41091504</t>
+        </is>
+      </c>
+      <c r="B517" t="inlineStr">
+        <is>
+          <t>What type of samples were sequenced?</t>
+        </is>
+      </c>
+      <c r="C517" t="inlineStr">
+        <is>
+          <t>PR</t>
+        </is>
+      </c>
+      <c r="D517" t="inlineStr"/>
+      <c r="E517" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="518">
+      <c r="A518" t="inlineStr">
+        <is>
+          <t>41093949</t>
+        </is>
+      </c>
+      <c r="B518" t="inlineStr">
+        <is>
+          <t>Does the paper report in vitro drug susceptibility data?</t>
+        </is>
+      </c>
+      <c r="C518" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D518" t="inlineStr"/>
+      <c r="E518" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="519">
+      <c r="A519" t="inlineStr">
+        <is>
+          <t>41093949</t>
+        </is>
+      </c>
+      <c r="B519" t="inlineStr">
+        <is>
+          <t>What were the GenBank accession numbers for sequenced HIV isolates?</t>
+        </is>
+      </c>
+      <c r="C519" t="inlineStr">
+        <is>
+          <t>Yes (recombinant clones)</t>
+        </is>
+      </c>
+      <c r="D519" t="inlineStr"/>
+      <c r="E519" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="520">
+      <c r="A520" t="inlineStr">
+        <is>
+          <t>41093949</t>
+        </is>
+      </c>
+      <c r="B520" t="inlineStr">
+        <is>
+          <t>Which HIV genes were reported to have been sequenced?</t>
+        </is>
+      </c>
+      <c r="C520" t="inlineStr">
+        <is>
+          <t>PQ735970–PQ735985</t>
+        </is>
+      </c>
+      <c r="D520" t="inlineStr"/>
+      <c r="E520" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="521">
+      <c r="A521" t="inlineStr">
+        <is>
+          <t>41093949</t>
+        </is>
+      </c>
+      <c r="B521" t="inlineStr">
+        <is>
+          <t>Were samples cloned prior to sequencing?</t>
+        </is>
+      </c>
+      <c r="C521" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D521" t="inlineStr"/>
+      <c r="E521" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="522">
+      <c r="A522" t="inlineStr">
+        <is>
+          <t>41093949</t>
+        </is>
+      </c>
+      <c r="B522" t="inlineStr">
+        <is>
+          <t>What type of samples were sequenced?</t>
+        </is>
+      </c>
+      <c r="C522" t="inlineStr">
+        <is>
+          <t>RT</t>
+        </is>
+      </c>
+      <c r="D522" t="inlineStr"/>
+      <c r="E522" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="523">
+      <c r="A523" t="inlineStr">
+        <is>
+          <t>41112839</t>
+        </is>
+      </c>
+      <c r="B523" t="inlineStr">
+        <is>
+          <t>Does the paper report HIV sequences from patient samples?</t>
+        </is>
+      </c>
+      <c r="C523" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D523" t="inlineStr"/>
+      <c r="E523" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="524">
+      <c r="A524" t="inlineStr">
+        <is>
+          <t>41112839</t>
+        </is>
+      </c>
+      <c r="B524" t="inlineStr">
+        <is>
+          <t>What were the GenBank accession numbers for sequenced HIV isolates?</t>
+        </is>
+      </c>
+      <c r="C524" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D524" t="inlineStr"/>
+      <c r="E524" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="525">
+      <c r="A525" t="inlineStr">
+        <is>
+          <t>41112839</t>
+        </is>
+      </c>
+      <c r="B525" t="inlineStr">
+        <is>
+          <t>Which HIV genes were reported to have been sequenced?</t>
+        </is>
+      </c>
+      <c r="C525" t="inlineStr">
+        <is>
+          <t>PP280627- PP280757</t>
+        </is>
+      </c>
+      <c r="D525" t="inlineStr"/>
+      <c r="E525" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="526">
+      <c r="A526" t="inlineStr">
+        <is>
+          <t>41112839</t>
+        </is>
+      </c>
+      <c r="B526" t="inlineStr">
+        <is>
+          <t>From which countries were the sequenced samples obtained?</t>
+        </is>
+      </c>
+      <c r="C526" t="inlineStr">
+        <is>
+          <t>237</t>
+        </is>
+      </c>
+      <c r="D526" t="inlineStr"/>
+      <c r="E526" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="527">
+      <c r="A527" t="inlineStr">
+        <is>
+          <t>41112839</t>
+        </is>
+      </c>
+      <c r="B527" t="inlineStr">
+        <is>
+          <t>From what years were the sequenced samples obtained?</t>
+        </is>
+      </c>
+      <c r="C527" t="inlineStr">
+        <is>
+          <t>Senegal</t>
+        </is>
+      </c>
+      <c r="D527" t="inlineStr"/>
+      <c r="E527" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="528">
+      <c r="A528" t="inlineStr">
+        <is>
+          <t>41112839</t>
+        </is>
+      </c>
+      <c r="B528" t="inlineStr">
+        <is>
+          <t>What method was used for sequencing?</t>
+        </is>
+      </c>
+      <c r="C528" t="inlineStr">
+        <is>
+          <t>2017-2018</t>
+        </is>
+      </c>
+      <c r="D528" t="inlineStr"/>
+      <c r="E528" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="529">
+      <c r="A529" t="inlineStr">
+        <is>
+          <t>41112839</t>
+        </is>
+      </c>
+      <c r="B529" t="inlineStr">
+        <is>
+          <t>What type of samples were sequenced?</t>
+        </is>
+      </c>
+      <c r="C529" t="inlineStr">
+        <is>
+          <t>RT</t>
+        </is>
+      </c>
+      <c r="D529" t="inlineStr"/>
+      <c r="E529" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="530">
+      <c r="A530" t="inlineStr">
+        <is>
+          <t>41129268</t>
+        </is>
+      </c>
+      <c r="B530" t="inlineStr">
+        <is>
+          <t>Does the paper report HIV sequences from patient samples?</t>
+        </is>
+      </c>
+      <c r="C530" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D530" t="inlineStr"/>
+      <c r="E530" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="531">
+      <c r="A531" t="inlineStr">
+        <is>
+          <t>41129268</t>
+        </is>
+      </c>
+      <c r="B531" t="inlineStr">
+        <is>
+          <t>From which countries were the sequenced samples obtained?</t>
+        </is>
+      </c>
+      <c r="C531" t="inlineStr">
+        <is>
+          <t>333</t>
+        </is>
+      </c>
+      <c r="D531" t="inlineStr"/>
+      <c r="E531" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="532">
+      <c r="A532" t="inlineStr">
+        <is>
+          <t>41129268</t>
+        </is>
+      </c>
+      <c r="B532" t="inlineStr">
+        <is>
+          <t>From what years were the sequenced samples obtained?</t>
+        </is>
+      </c>
+      <c r="C532" t="inlineStr">
+        <is>
+          <t>Uganda</t>
+        </is>
+      </c>
+      <c r="D532" t="inlineStr"/>
+      <c r="E532" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="533">
+      <c r="A533" t="inlineStr">
+        <is>
+          <t>41129268</t>
+        </is>
+      </c>
+      <c r="B533" t="inlineStr">
+        <is>
+          <t>What method was used for sequencing?</t>
+        </is>
+      </c>
+      <c r="C533" t="inlineStr">
+        <is>
+          <t>2021</t>
+        </is>
+      </c>
+      <c r="D533" t="inlineStr"/>
+      <c r="E533" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="534">
+      <c r="A534" t="inlineStr">
+        <is>
+          <t>41129268</t>
+        </is>
+      </c>
+      <c r="B534" t="inlineStr">
+        <is>
+          <t>What type of samples were sequenced?</t>
+        </is>
+      </c>
+      <c r="C534" t="inlineStr">
+        <is>
+          <t>RT, PR, IN</t>
+        </is>
+      </c>
+      <c r="D534" t="inlineStr"/>
+      <c r="E534" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="535">
+      <c r="A535" t="inlineStr">
+        <is>
+          <t>41129268</t>
+        </is>
+      </c>
+      <c r="B535" t="inlineStr">
+        <is>
+          <t>How many individuals had samples obtained for HIV sequencing?</t>
+        </is>
+      </c>
+      <c r="C535" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D535" t="inlineStr"/>
+      <c r="E535" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="536">
+      <c r="A536" t="inlineStr">
+        <is>
+          <t>41129268</t>
+        </is>
+      </c>
+      <c r="B536" t="inlineStr">
+        <is>
+          <t>Which drug classes were received by individuals in the study before sample sequencing?</t>
+        </is>
+      </c>
+      <c r="C536" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D536" t="inlineStr"/>
+      <c r="E536" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="537">
+      <c r="A537" t="inlineStr">
+        <is>
+          <t>41129268</t>
+        </is>
+      </c>
+      <c r="B537" t="inlineStr">
+        <is>
+          <t>Which drugs were received by individuals in the study before sample sequencing?</t>
+        </is>
+      </c>
+      <c r="C537" t="inlineStr">
+        <is>
+          <t>NRTI, NNRTI, PI, INSTI</t>
+        </is>
+      </c>
+      <c r="D537" t="inlineStr"/>
+      <c r="E537" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="538">
+      <c r="A538" t="inlineStr">
+        <is>
+          <t>41130593</t>
+        </is>
+      </c>
+      <c r="B538" t="inlineStr">
+        <is>
+          <t>Does the paper report HIV sequences from patient samples?</t>
+        </is>
+      </c>
+      <c r="C538" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D538" t="inlineStr"/>
+      <c r="E538" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="539">
+      <c r="A539" t="inlineStr">
+        <is>
+          <t>41130593</t>
+        </is>
+      </c>
+      <c r="B539" t="inlineStr">
+        <is>
+          <t>From which countries were the sequenced samples obtained?</t>
+        </is>
+      </c>
+      <c r="C539" t="inlineStr">
+        <is>
+          <t>64</t>
+        </is>
+      </c>
+      <c r="D539" t="inlineStr"/>
+      <c r="E539" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="540">
+      <c r="A540" t="inlineStr">
+        <is>
+          <t>41130593</t>
+        </is>
+      </c>
+      <c r="B540" t="inlineStr">
+        <is>
+          <t>Were samples cloned prior to sequencing?</t>
+        </is>
+      </c>
+      <c r="C540" t="inlineStr">
+        <is>
+          <t>Yes (single genome)</t>
+        </is>
+      </c>
+      <c r="D540" t="inlineStr"/>
+      <c r="E540" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="541">
+      <c r="A541" t="inlineStr">
+        <is>
+          <t>41130593</t>
+        </is>
+      </c>
+      <c r="B541" t="inlineStr">
+        <is>
+          <t>What type of samples were sequenced?</t>
+        </is>
+      </c>
+      <c r="C541" t="inlineStr">
+        <is>
+          <t>RT,PR,IN,CA</t>
+        </is>
+      </c>
+      <c r="D541" t="inlineStr"/>
+      <c r="E541" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="542">
+      <c r="A542" t="inlineStr">
+        <is>
+          <t>41130593</t>
+        </is>
+      </c>
+      <c r="B542" t="inlineStr">
+        <is>
+          <t>How many individuals had samples obtained for HIV sequencing?</t>
+        </is>
+      </c>
+      <c r="C542" t="inlineStr">
+        <is>
+          <t>Yes (PrEP)</t>
+        </is>
+      </c>
+      <c r="D542" t="inlineStr"/>
+      <c r="E542" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="543">
+      <c r="A543" t="inlineStr">
+        <is>
+          <t>41130593</t>
+        </is>
+      </c>
+      <c r="B543" t="inlineStr">
+        <is>
+          <t>Does the paper report HIV sequences from individuals who had previously received ARV drugs?</t>
+        </is>
+      </c>
+      <c r="C543" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D543" t="inlineStr"/>
+      <c r="E543" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="544">
+      <c r="A544" t="inlineStr">
+        <is>
+          <t>41130593</t>
+        </is>
+      </c>
+      <c r="B544" t="inlineStr">
+        <is>
+          <t>Which drug classes were received by individuals in the study before sample sequencing?</t>
+        </is>
+      </c>
+      <c r="C544" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D544" t="inlineStr"/>
+      <c r="E544" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="545">
+      <c r="A545" t="inlineStr">
+        <is>
+          <t>41130593</t>
+        </is>
+      </c>
+      <c r="B545" t="inlineStr">
+        <is>
+          <t>Which drugs were received by individuals in the study before sample sequencing?</t>
+        </is>
+      </c>
+      <c r="C545" t="inlineStr">
+        <is>
+          <t>NRTI, CAI</t>
+        </is>
+      </c>
+      <c r="D545" t="inlineStr"/>
+      <c r="E545" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="546">
+      <c r="A546" t="inlineStr">
+        <is>
+          <t>41140464</t>
+        </is>
+      </c>
+      <c r="B546" t="inlineStr">
+        <is>
+          <t>From what years were the sequenced samples obtained?</t>
+        </is>
+      </c>
+      <c r="C546" t="inlineStr">
+        <is>
+          <t>Tanzania</t>
+        </is>
+      </c>
+      <c r="D546" t="inlineStr"/>
+      <c r="E546" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="547">
+      <c r="A547" t="inlineStr">
+        <is>
+          <t>41140464</t>
+        </is>
+      </c>
+      <c r="B547" t="inlineStr">
+        <is>
+          <t>What type of samples were sequenced?</t>
+        </is>
+      </c>
+      <c r="C547" t="inlineStr">
+        <is>
+          <t>PR, RT, IN</t>
+        </is>
+      </c>
+      <c r="D547" t="inlineStr"/>
+      <c r="E547" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="548">
+      <c r="A548" t="inlineStr">
+        <is>
+          <t>41140464</t>
+        </is>
+      </c>
+      <c r="B548" t="inlineStr">
+        <is>
+          <t>How many individuals had samples obtained for HIV sequencing?</t>
+        </is>
+      </c>
+      <c r="C548" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D548" t="inlineStr"/>
+      <c r="E548" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="549">
+      <c r="A549" t="inlineStr">
+        <is>
+          <t>41140464</t>
+        </is>
+      </c>
+      <c r="B549" t="inlineStr">
+        <is>
+          <t>Which drug classes were received by individuals in the study before sample sequencing?</t>
+        </is>
+      </c>
+      <c r="C549" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D549" t="inlineStr"/>
+      <c r="E549" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="550">
+      <c r="A550" t="inlineStr">
+        <is>
+          <t>41140464</t>
+        </is>
+      </c>
+      <c r="B550" t="inlineStr">
+        <is>
+          <t>Which drugs were received by individuals in the study before sample sequencing?</t>
+        </is>
+      </c>
+      <c r="C550" t="inlineStr">
+        <is>
+          <t>NRTI, NNRTI, PI, INSTI</t>
+        </is>
+      </c>
+      <c r="D550" t="inlineStr"/>
+      <c r="E550" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>